<commit_message>
Updated and modified the version
</commit_message>
<xml_diff>
--- a/injectionlist/Sample Submission Example.xlsx
+++ b/injectionlist/Sample Submission Example.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C0D9D69-13E2-4951-9C22-CD403CADA36F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{CEA36611-A8E5-D14A-A501-7AD91DE4C3CC}"/>
+    <workbookView xWindow="3780" yWindow="2520" windowWidth="19200" windowHeight="11250" xr2:uid="{CEA36611-A8E5-D14A-A501-7AD91DE4C3CC}"/>
   </bookViews>
   <sheets>
     <sheet name="SampleSubmissionForm" sheetId="1" r:id="rId1"/>
@@ -29987,9 +29987,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -30131,26 +30134,15 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CFCFC8B2-EA4C-46FD-A6B9-7938CFB57E38}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C504CC50-8BC5-4D63-8FB8-BA0342AD8B37}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="b184d495-6532-4d88-9e37-ac7f4182d535"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -30174,9 +30166,17 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C504CC50-8BC5-4D63-8FB8-BA0342AD8B37}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CFCFC8B2-EA4C-46FD-A6B9-7938CFB57E38}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="b184d495-6532-4d88-9e37-ac7f4182d535"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>